<commit_message>
developing tests on incoming data
</commit_message>
<xml_diff>
--- a/borough_template.xlsx
+++ b/borough_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Teams\D&amp;PA\Apps\Local Elections\1 - Collect results\produce_from\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D31D4024-EA2B-4FAB-AD04-9C5AD42A9924}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC437DA0-F4D9-4135-8924-AA68828FCAFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="23657" windowHeight="15240" tabRatio="890" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t>Report of Election for the Greater London Authority</t>
   </si>
@@ -71,7 +71,7 @@
     <t>Ballot papers from postal votes</t>
   </si>
   <si>
-    <t>Percentage poll</t>
+    <t>Turnout</t>
   </si>
   <si>
     <t>Total number of rejected ballot papers</t>
@@ -101,10 +101,7 @@
     <t>First name</t>
   </si>
   <si>
-    <t>Initials</t>
-  </si>
-  <si>
-    <t>Whether Female</t>
+    <t>Whether Female (if known)</t>
   </si>
   <si>
     <t>Party</t>
@@ -252,7 +249,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -289,17 +286,6 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="22"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top/>
       <bottom style="thin">
         <color indexed="22"/>
@@ -401,7 +387,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -427,9 +413,6 @@
     <xf numFmtId="3" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="2" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -454,6 +437,9 @@
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -467,9 +453,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -841,38 +824,38 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:I40"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.1"/>
+  <dimension ref="A1:I44"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="3.42578125" style="15" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" style="14" customWidth="1"/>
     <col min="2" max="2" width="20.42578125" style="1" customWidth="1"/>
     <col min="3" max="3" width="12.140625" style="1" customWidth="1"/>
-    <col min="4" max="4" width="7.85546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="22.7109375" style="1" customWidth="1"/>
     <col min="5" max="5" width="18.5703125" style="1" customWidth="1"/>
     <col min="6" max="6" width="32.7109375" style="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7109375" style="10" customWidth="1"/>
+    <col min="7" max="7" width="29.140625" style="10" customWidth="1"/>
     <col min="8" max="8" width="26.5703125" style="3" customWidth="1"/>
-    <col min="9" max="9" width="29.28515625" style="18" customWidth="1"/>
+    <col min="9" max="9" width="29.28515625" style="17" customWidth="1"/>
     <col min="10" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.4">
-      <c r="A1" s="17" t="s">
+    <row r="1" spans="1:9" ht="15.75">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="20.25" customHeight="1">
-      <c r="A3" s="13" t="s">
+    <row r="3" spans="1:9" ht="15">
+      <c r="A3" s="12" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="21.75" customHeight="1">
-      <c r="A4" s="14" t="s">
+    <row r="4" spans="1:9">
+      <c r="A4" s="13" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="8"/>
@@ -880,13 +863,10 @@
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
-      <c r="G4" s="11"/>
-      <c r="H4" s="26">
-        <v>43956</v>
-      </c>
+      <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:9">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="13" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="8"/>
@@ -894,14 +874,13 @@
       <c r="D5" s="8"/>
       <c r="E5" s="8"/>
       <c r="F5" s="8"/>
-      <c r="G5" s="11"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="18" t="s">
+      <c r="G5" s="26"/>
+      <c r="I5" s="17" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:9">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="13" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="8"/>
@@ -909,11 +888,10 @@
       <c r="D6" s="8"/>
       <c r="E6" s="8"/>
       <c r="F6" s="8"/>
-      <c r="G6" s="11"/>
-      <c r="H6" s="27"/>
+      <c r="G6" s="26"/>
     </row>
     <row r="7" spans="1:9">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="8"/>
@@ -921,11 +899,10 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="11"/>
-      <c r="H7" s="27"/>
-    </row>
-    <row r="8" spans="1:9" ht="27.75" customHeight="1">
-      <c r="A8" s="14" t="s">
+      <c r="G7" s="26"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="13" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="8"/>
@@ -933,11 +910,10 @@
       <c r="D8" s="8"/>
       <c r="E8" s="8"/>
       <c r="F8" s="8"/>
-      <c r="G8" s="11"/>
-      <c r="H8" s="4"/>
+      <c r="G8" s="4"/>
     </row>
     <row r="9" spans="1:9">
-      <c r="A9" s="14"/>
+      <c r="A9" s="13"/>
       <c r="B9" s="8" t="s">
         <v>9</v>
       </c>
@@ -945,11 +921,10 @@
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
-      <c r="G9" s="11"/>
-      <c r="H9" s="4"/>
+      <c r="G9" s="4"/>
     </row>
     <row r="10" spans="1:9">
-      <c r="A10" s="14"/>
+      <c r="A10" s="13"/>
       <c r="B10" s="8" t="s">
         <v>10</v>
       </c>
@@ -957,11 +932,10 @@
       <c r="D10" s="8"/>
       <c r="E10" s="8"/>
       <c r="F10" s="8"/>
-      <c r="G10" s="11"/>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:9" ht="21" customHeight="1">
-      <c r="A11" s="14"/>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="13"/>
       <c r="B11" s="8" t="s">
         <v>11</v>
       </c>
@@ -969,11 +943,10 @@
       <c r="D11" s="8"/>
       <c r="E11" s="8"/>
       <c r="F11" s="8"/>
-      <c r="G11" s="11"/>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:9" ht="25.5" customHeight="1">
-      <c r="A12" s="14" t="s">
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="13" t="s">
         <v>12</v>
       </c>
       <c r="B12" s="8"/>
@@ -981,11 +954,10 @@
       <c r="D12" s="8"/>
       <c r="E12" s="8"/>
       <c r="F12" s="8"/>
-      <c r="G12" s="11"/>
-      <c r="H12" s="4"/>
+      <c r="G12" s="4"/>
     </row>
     <row r="13" spans="1:9">
-      <c r="A13" s="14"/>
+      <c r="A13" s="13"/>
       <c r="B13" s="8" t="s">
         <v>13</v>
       </c>
@@ -993,11 +965,10 @@
       <c r="D13" s="8"/>
       <c r="E13" s="8"/>
       <c r="F13" s="8"/>
-      <c r="G13" s="11"/>
-      <c r="H13" s="4"/>
+      <c r="G13" s="4"/>
     </row>
     <row r="14" spans="1:9">
-      <c r="A14" s="14"/>
+      <c r="A14" s="13"/>
       <c r="B14" s="8" t="s">
         <v>14</v>
       </c>
@@ -1005,11 +976,10 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="8"/>
-      <c r="G14" s="11"/>
-      <c r="H14" s="4"/>
+      <c r="G14" s="4"/>
     </row>
     <row r="15" spans="1:9">
-      <c r="A15" s="14"/>
+      <c r="A15" s="13"/>
       <c r="B15" s="8" t="s">
         <v>15</v>
       </c>
@@ -1017,11 +987,10 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="8"/>
-      <c r="G15" s="11"/>
-      <c r="H15" s="4"/>
+      <c r="G15" s="4"/>
     </row>
     <row r="16" spans="1:9">
-      <c r="A16" s="14"/>
+      <c r="A16" s="13"/>
       <c r="B16" s="8" t="s">
         <v>16</v>
       </c>
@@ -1029,11 +998,10 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="8"/>
-      <c r="G16" s="11"/>
-      <c r="H16" s="4"/>
-    </row>
-    <row r="17" spans="1:9" ht="22.5" customHeight="1">
-      <c r="A17" s="14" t="s">
+      <c r="G16" s="4"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="13" t="s">
         <v>17</v>
       </c>
       <c r="B17" s="8"/>
@@ -1041,16 +1009,15 @@
       <c r="D17" s="8"/>
       <c r="E17" s="8"/>
       <c r="F17" s="8"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="4"/>
-    </row>
-    <row r="18" spans="1:9" ht="37.5" customHeight="1">
+      <c r="G17" s="4"/>
+    </row>
+    <row r="18" spans="1:9" ht="15">
       <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
     </row>
     <row r="19" spans="1:9" s="7" customFormat="1" ht="28.5">
-      <c r="A19" s="16"/>
+      <c r="A19" s="15"/>
       <c r="B19" s="5" t="s">
         <v>19</v>
       </c>
@@ -1063,336 +1030,357 @@
       <c r="E19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F19" s="5" t="s">
+      <c r="F19" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="9" t="s">
+      <c r="G19" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="H19" s="6" t="s">
+      <c r="H19" s="18"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="14">
+        <v>1</v>
+      </c>
+      <c r="B20" s="19"/>
+      <c r="C20" s="20"/>
+      <c r="D20" s="20"/>
+      <c r="E20" s="21"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="17" t="s">
         <v>25</v>
       </c>
-      <c r="I19" s="19"/>
-    </row>
-    <row r="20" spans="1:9" ht="15.75" customHeight="1">
-      <c r="A20" s="15">
-        <v>1</v>
-      </c>
-      <c r="B20" s="20"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="21"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="18" t="s">
+      <c r="I20" s="1"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="14">
+        <v>2</v>
+      </c>
+      <c r="B21" s="22"/>
+      <c r="C21" s="23"/>
+      <c r="D21" s="23"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="24"/>
+      <c r="G21" s="24"/>
+      <c r="H21" s="17" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="15">
-        <v>2</v>
-      </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
-      <c r="I21" s="18" t="s">
+      <c r="I21" s="1"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="14">
+        <v>3</v>
+      </c>
+      <c r="B22" s="22"/>
+      <c r="C22" s="23"/>
+      <c r="D22" s="23"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="24"/>
+      <c r="G22" s="24"/>
+      <c r="H22" s="17" t="s">
         <v>27</v>
       </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="15">
-        <v>3</v>
-      </c>
-      <c r="B22" s="23"/>
-      <c r="C22" s="24"/>
-      <c r="D22" s="24"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="25"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="25"/>
-      <c r="I22" s="18" t="s">
+      <c r="I22" s="1"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="14">
+        <v>4</v>
+      </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="23"/>
+      <c r="D23" s="23"/>
+      <c r="E23" s="24"/>
+      <c r="F23" s="24"/>
+      <c r="G23" s="24"/>
+      <c r="H23" s="17" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" s="15">
-        <v>4</v>
-      </c>
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="24"/>
-      <c r="F23" s="25"/>
-      <c r="G23" s="25"/>
-      <c r="H23" s="25"/>
-      <c r="I23" s="18" t="s">
+      <c r="I23" s="1"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="14">
+        <v>5</v>
+      </c>
+      <c r="B24" s="22"/>
+      <c r="C24" s="23"/>
+      <c r="D24" s="23"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
+      <c r="H24" s="17" t="s">
         <v>29</v>
       </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" s="15">
-        <v>5</v>
-      </c>
-      <c r="B24" s="23"/>
-      <c r="C24" s="24"/>
-      <c r="D24" s="24"/>
-      <c r="E24" s="24"/>
-      <c r="F24" s="25"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="25"/>
-      <c r="I24" s="18" t="s">
+      <c r="I24" s="1"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="14">
+        <v>6</v>
+      </c>
+      <c r="B25" s="22"/>
+      <c r="C25" s="23"/>
+      <c r="D25" s="23"/>
+      <c r="E25" s="24"/>
+      <c r="F25" s="24"/>
+      <c r="G25" s="24"/>
+      <c r="H25" s="17" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" s="15">
-        <v>6</v>
-      </c>
-      <c r="B25" s="23"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="25"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="25"/>
-      <c r="I25" s="18" t="s">
+      <c r="I25" s="1"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="14">
+        <v>7</v>
+      </c>
+      <c r="B26" s="22"/>
+      <c r="C26" s="23"/>
+      <c r="D26" s="23"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="24"/>
+      <c r="G26" s="24"/>
+      <c r="H26" s="17" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" s="15">
-        <v>7</v>
-      </c>
-      <c r="B26" s="23"/>
-      <c r="C26" s="24"/>
-      <c r="D26" s="24"/>
-      <c r="E26" s="24"/>
-      <c r="F26" s="25"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="25"/>
-      <c r="I26" s="18" t="s">
+      <c r="I26" s="1"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="14">
+        <v>8</v>
+      </c>
+      <c r="B27" s="22"/>
+      <c r="C27" s="23"/>
+      <c r="D27" s="23"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="24"/>
+      <c r="G27" s="24"/>
+      <c r="H27" s="17" t="s">
         <v>32</v>
       </c>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27" s="15">
-        <v>8</v>
-      </c>
-      <c r="B27" s="23"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="25"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="25"/>
-      <c r="I27" s="18" t="s">
+      <c r="I27" s="1"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="14">
+        <v>9</v>
+      </c>
+      <c r="B28" s="22"/>
+      <c r="C28" s="23"/>
+      <c r="D28" s="23"/>
+      <c r="E28" s="24"/>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="17" t="s">
         <v>33</v>
       </c>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28" s="15">
-        <v>9</v>
-      </c>
-      <c r="B28" s="23"/>
-      <c r="C28" s="24"/>
-      <c r="D28" s="24"/>
-      <c r="E28" s="24"/>
-      <c r="F28" s="25"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="25"/>
-      <c r="I28" s="18" t="s">
+      <c r="I28" s="1"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="14">
+        <v>10</v>
+      </c>
+      <c r="B29" s="22"/>
+      <c r="C29" s="23"/>
+      <c r="D29" s="23"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="24"/>
+      <c r="G29" s="24"/>
+      <c r="H29" s="17" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" s="15">
-        <v>10</v>
-      </c>
-      <c r="B29" s="23"/>
-      <c r="C29" s="24"/>
-      <c r="D29" s="24"/>
-      <c r="E29" s="24"/>
-      <c r="F29" s="25"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="25"/>
-      <c r="I29" s="18" t="s">
+      <c r="I29" s="1"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="14">
+        <v>11</v>
+      </c>
+      <c r="B30" s="22"/>
+      <c r="C30" s="23"/>
+      <c r="D30" s="23"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="24"/>
+      <c r="G30" s="24"/>
+      <c r="H30" s="17" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="30" spans="1:9">
-      <c r="A30" s="15">
-        <v>11</v>
-      </c>
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="18" t="s">
+      <c r="I30" s="1"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="14">
+        <v>12</v>
+      </c>
+      <c r="B31" s="22"/>
+      <c r="C31" s="23"/>
+      <c r="D31" s="23"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="24"/>
+      <c r="G31" s="24"/>
+      <c r="H31" s="17" t="s">
         <v>36</v>
       </c>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="A31" s="15">
-        <v>12</v>
-      </c>
-      <c r="B31" s="23"/>
-      <c r="C31" s="24"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="25"/>
-      <c r="I31" s="18" t="s">
+      <c r="I31" s="1"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="14">
+        <v>13</v>
+      </c>
+      <c r="B32" s="22"/>
+      <c r="C32" s="23"/>
+      <c r="D32" s="23"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="24"/>
+      <c r="G32" s="24"/>
+      <c r="H32" s="17" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="A32" s="15">
-        <v>13</v>
-      </c>
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="25"/>
-      <c r="H32" s="25"/>
-      <c r="I32" s="18" t="s">
+      <c r="I32" s="1"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="14">
+        <v>14</v>
+      </c>
+      <c r="B33" s="22"/>
+      <c r="C33" s="23"/>
+      <c r="D33" s="23"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="24"/>
+      <c r="G33" s="24"/>
+      <c r="H33" s="17" t="s">
         <v>38</v>
       </c>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" s="15">
-        <v>14</v>
-      </c>
-      <c r="B33" s="23"/>
-      <c r="C33" s="24"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="25"/>
-      <c r="I33" s="18" t="s">
+      <c r="I33" s="1"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="14">
+        <v>15</v>
+      </c>
+      <c r="B34" s="22"/>
+      <c r="C34" s="23"/>
+      <c r="D34" s="23"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="24"/>
+      <c r="G34" s="24"/>
+      <c r="H34" s="17" t="s">
         <v>39</v>
       </c>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="A34" s="15">
-        <v>15</v>
-      </c>
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
-      <c r="I34" s="18" t="s">
+      <c r="I34" s="1"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="14">
+        <v>16</v>
+      </c>
+      <c r="B35" s="22"/>
+      <c r="C35" s="23"/>
+      <c r="D35" s="23"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="24"/>
+      <c r="G35" s="24"/>
+      <c r="H35" s="17" t="s">
         <v>40</v>
       </c>
-    </row>
-    <row r="35" spans="1:9">
-      <c r="A35" s="15">
-        <v>16</v>
-      </c>
-      <c r="B35" s="23"/>
-      <c r="C35" s="24"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="25"/>
-      <c r="H35" s="25"/>
-      <c r="I35" s="18" t="s">
+      <c r="I35" s="1"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="14">
+        <v>17</v>
+      </c>
+      <c r="B36" s="22"/>
+      <c r="C36" s="23"/>
+      <c r="D36" s="23"/>
+      <c r="E36" s="24"/>
+      <c r="F36" s="24"/>
+      <c r="G36" s="24"/>
+      <c r="H36" s="17" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" s="15">
-        <v>17</v>
-      </c>
-      <c r="B36" s="23"/>
-      <c r="C36" s="24"/>
-      <c r="D36" s="24"/>
-      <c r="E36" s="24"/>
-      <c r="F36" s="25"/>
-      <c r="G36" s="25"/>
-      <c r="H36" s="25"/>
-      <c r="I36" s="18" t="s">
+      <c r="I36" s="1"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="14">
+        <v>18</v>
+      </c>
+      <c r="B37" s="22"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="24"/>
+      <c r="F37" s="24"/>
+      <c r="G37" s="24"/>
+      <c r="H37" s="17" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" s="15">
-        <v>18</v>
-      </c>
-      <c r="B37" s="23"/>
-      <c r="C37" s="24"/>
-      <c r="D37" s="24"/>
-      <c r="E37" s="24"/>
-      <c r="F37" s="25"/>
-      <c r="G37" s="25"/>
-      <c r="H37" s="25"/>
-      <c r="I37" s="18" t="s">
+      <c r="I37" s="1"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="14">
+        <v>19</v>
+      </c>
+      <c r="B38" s="22"/>
+      <c r="C38" s="23"/>
+      <c r="D38" s="23"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="24"/>
+      <c r="G38" s="24"/>
+      <c r="H38" s="17" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" s="15">
-        <v>19</v>
-      </c>
-      <c r="B38" s="23"/>
-      <c r="C38" s="24"/>
-      <c r="D38" s="24"/>
-      <c r="E38" s="24"/>
-      <c r="F38" s="25"/>
-      <c r="G38" s="25"/>
-      <c r="H38" s="25"/>
-      <c r="I38" s="18" t="s">
+      <c r="I38" s="1"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="14">
+        <v>20</v>
+      </c>
+      <c r="B39" s="22"/>
+      <c r="C39" s="23"/>
+      <c r="D39" s="23"/>
+      <c r="E39" s="24"/>
+      <c r="F39" s="24"/>
+      <c r="G39" s="24"/>
+      <c r="H39" s="17" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="39" spans="1:9">
-      <c r="A39" s="15">
-        <v>20</v>
-      </c>
-      <c r="B39" s="23"/>
-      <c r="C39" s="24"/>
-      <c r="D39" s="24"/>
-      <c r="E39" s="24"/>
-      <c r="F39" s="25"/>
-      <c r="G39" s="25"/>
-      <c r="H39" s="25"/>
-      <c r="I39" s="18" t="s">
+      <c r="I39" s="1"/>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="14">
+        <v>21</v>
+      </c>
+      <c r="B40" s="22"/>
+      <c r="C40" s="23"/>
+      <c r="D40" s="23"/>
+      <c r="E40" s="24"/>
+      <c r="F40" s="24"/>
+      <c r="G40" s="24"/>
+      <c r="H40" s="17" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="40" spans="1:9">
-      <c r="A40" s="15">
-        <v>21</v>
-      </c>
-      <c r="B40" s="23"/>
-      <c r="C40" s="24"/>
-      <c r="D40" s="24"/>
-      <c r="E40" s="24"/>
-      <c r="F40" s="25"/>
-      <c r="G40" s="25"/>
-      <c r="H40" s="25"/>
-      <c r="I40" s="18" t="s">
-        <v>46</v>
-      </c>
+      <c r="I40" s="1"/>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="F41" s="10"/>
+      <c r="G41" s="3"/>
+      <c r="H41" s="17"/>
+      <c r="I41" s="1"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="F42" s="10"/>
+      <c r="G42" s="3"/>
+      <c r="H42" s="17"/>
+      <c r="I42" s="1"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="F43" s="10"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="17"/>
+      <c r="I43" s="1"/>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="F44" s="10"/>
+      <c r="G44" s="3"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="1"/>
     </row>
   </sheetData>
   <dataConsolidate/>
   <phoneticPr fontId="2" type="noConversion"/>
-  <conditionalFormatting sqref="B20:F40">
+  <conditionalFormatting sqref="B20:E40">
     <cfRule type="expression" dxfId="7" priority="7" stopIfTrue="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -1408,7 +1396,7 @@
       <formula>MOD(ROW(),2)=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G20:G40">
+  <conditionalFormatting sqref="F20:F40">
     <cfRule type="expression" dxfId="3" priority="3" stopIfTrue="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
@@ -1416,7 +1404,7 @@
       <formula>MOD(ROW(),2)=1</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H20:H40">
+  <conditionalFormatting sqref="G20:G40">
     <cfRule type="expression" dxfId="1" priority="1" stopIfTrue="1">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>

</xml_diff>